<commit_message>
New logo test files
</commit_message>
<xml_diff>
--- a/awyiss/Command/Media/TestFiles/logo-awyiss.xlsx
+++ b/awyiss/Command/Media/TestFiles/logo-awyiss.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabsn182\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\cms\awyiss\Command\Media\TestFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{465394CA-0895-4CB1-A74A-C388F12F0711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518B2F39-4309-427E-A6C6-2A05D18433D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4455" yWindow="5190" windowWidth="28800" windowHeight="15375" xr2:uid="{AE7ED264-6765-46C3-80B8-5D657B262B1F}"/>
+    <workbookView xWindow="4800" yWindow="5235" windowWidth="27330" windowHeight="15090" xr2:uid="{AE7ED264-6765-46C3-80B8-5D657B262B1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -272,74 +272,56 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>3</xdr:col>
-          <xdr:colOff>95250</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>85725</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>9</xdr:col>
-          <xdr:colOff>676275</xdr:colOff>
-          <xdr:row>20</xdr:row>
-          <xdr:rowOff>66675</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1025" name="Object 1" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1025"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94A4D82A-9506-05EC-1CA7-AAB8462AE12E}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-            </a:solidFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd type="none" w="med" len="med"/>
-            </a:ln>
-            <a:effectLst/>
-            <a:extLst>
-              <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-                <a14:hiddenEffects>
-                  <a:effectLst>
-                    <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="808080"/>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </a14:hiddenEffects>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>447675</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Grafik 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F83D22F-2864-A219-23AD-60F6D5FEF998}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2733675" y="1924050"/>
+          <a:ext cx="5095875" cy="1600200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -639,7 +621,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F31D50D-A138-47B6-BA37-0C268B3E0155}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F31D50D-A138-47B6-BA37-0C268B3E0155}">
   <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -827,33 +809,5 @@
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
-  <oleObjects>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <oleObject shapeId="1025" r:id="rId3">
-          <objectPr defaultSize="0" r:id="rId4">
-            <anchor moveWithCells="1">
-              <from>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>95250</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>85725</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>9</xdr:col>
-                <xdr:colOff>676275</xdr:colOff>
-                <xdr:row>20</xdr:row>
-                <xdr:rowOff>66675</xdr:rowOff>
-              </to>
-            </anchor>
-          </objectPr>
-        </oleObject>
-      </mc:Choice>
-      <mc:Fallback>
-        <oleObject shapeId="1025" r:id="rId3"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-  </oleObjects>
 </worksheet>
 </file>
</xml_diff>